<commit_message>
Corrected Aggregate tools and Metadata tools
</commit_message>
<xml_diff>
--- a/WorkFlow Genie/backend/data/excel_files/00e83810-7d86-4bfb-8983-a3732132aaa6_expense_sheet.xlsx
+++ b/WorkFlow Genie/backend/data/excel_files/00e83810-7d86-4bfb-8983-a3732132aaa6_expense_sheet.xlsx
@@ -2,22 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Pivot_Sheet1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,12 +23,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,35 +48,24 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -148,116 +135,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Amount Spent by Department</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Sheet1'!B1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Sheet1'!$A$2:$A$10</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Sheet1'!$B$2:$B$10</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5400000" cy="2700000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -335,6 +212,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -369,6 +247,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -403,20 +282,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -538,7 +413,46 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -549,8 +463,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E101"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E102"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -580,2508 +494,2333 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>EXP-0001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2025-05-19</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="B2" s="2" t="n">
+        <v>45796</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Server Hosting</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
         <v>998.37</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>EXP-0002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-02-13</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="B3" s="2" t="n">
+        <v>46066</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Internet Bill</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="2" t="n">
         <v>2704.61</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>EXP-0003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-03-30</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="B4" s="2" t="n">
+        <v>46111</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Airfare</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
         <v>743.9</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>EXP-0004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2025-11-22</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="B5" s="2" t="n">
+        <v>45983</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Pantry Supplies</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="2" t="n">
         <v>958.27</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>EXP-0005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2025-12-07</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+      <c r="B6" s="2" t="n">
+        <v>45998</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Online Ads</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="2" t="n">
         <v>2340.01</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>EXP-0006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2025-12-18</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="B7" s="2" t="n">
+        <v>46009</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Pantry Supplies</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="2" t="n">
         <v>4378.71</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>EXP-0007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-01-30</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="B8" s="2" t="n">
+        <v>46052</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Hotel Accommodation</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="2" t="n">
         <v>423.16</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>EXP-0008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-02-18</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="B9" s="2" t="n">
+        <v>46071</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Hotel Accommodation</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="2" t="n">
         <v>4049.71</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>EXP-0009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2025-04-30</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="B10" s="2" t="n">
+        <v>45777</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Legal Consultation</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="2" t="n">
         <v>4287.04</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>EXP-0010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2025-07-06</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
+      <c r="B11" s="2" t="n">
+        <v>45844</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Server Hosting</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="2" t="n">
         <v>534.65</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>EXP-0011</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-02-26</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="B12" s="2" t="n">
+        <v>46079</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Online Ads</t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="2" t="n">
         <v>3278.12</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>EXP-0012</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2025-06-13</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
+      <c r="B13" s="2" t="n">
+        <v>45821</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Hotel Accommodation</t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="2" t="n">
         <v>2725.91</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>EXP-0013</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2025-09-07</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
+      <c r="B14" s="2" t="n">
+        <v>45907</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Team Lunch</t>
         </is>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="2" t="n">
         <v>123.05</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>EXP-0014</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
+      <c r="B15" s="2" t="n">
+        <v>46107</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Online Ads</t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="2" t="n">
         <v>511.65</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>EXP-0015</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
+      <c r="B16" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Internet Bill</t>
         </is>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="2" t="n">
         <v>3780.15</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>EXP-0016</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+      <c r="B17" s="2" t="n">
+        <v>46076</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Event Sponsorship</t>
         </is>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="2" t="n">
         <v>1220.08</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>EXP-0017</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>2025-12-21</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
+      <c r="B18" s="2" t="n">
+        <v>46012</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Laptops</t>
         </is>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="2" t="n">
         <v>2061.75</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>EXP-0018</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2025-12-13</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
+      <c r="B19" s="2" t="n">
+        <v>46004</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="2" t="n">
         <v>2432.72</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>EXP-0019</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2025-07-27</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
+      <c r="B20" s="2" t="n">
+        <v>45865</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Electricity Bill</t>
         </is>
       </c>
-      <c r="E20" t="n">
+      <c r="E20" s="2" t="n">
         <v>4330.02</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>EXP-0020</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>2025-06-07</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
+      <c r="B21" s="2" t="n">
+        <v>45815</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Online Ads</t>
         </is>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="2" t="n">
         <v>4517.09</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>EXP-0021</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>2026-03-29</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
+      <c r="B22" s="2" t="n">
+        <v>46110</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Pantry Supplies</t>
         </is>
       </c>
-      <c r="E22" t="n">
+      <c r="E22" s="2" t="n">
         <v>864.95</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>EXP-0022</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2025-06-28</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
+      <c r="B23" s="2" t="n">
+        <v>45836</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Training Courses</t>
         </is>
       </c>
-      <c r="E23" t="n">
+      <c r="E23" s="2" t="n">
         <v>60.67</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>EXP-0023</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>2025-12-31</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
+      <c r="B24" s="2" t="n">
+        <v>46022</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Training Courses</t>
         </is>
       </c>
-      <c r="E24" t="n">
+      <c r="E24" s="2" t="n">
         <v>1982.59</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>EXP-0024</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>2025-05-14</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
+      <c r="B25" s="2" t="n">
+        <v>45791</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E25" t="n">
+      <c r="E25" s="2" t="n">
         <v>4636.26</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>EXP-0025</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>2025-04-17</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
+      <c r="B26" s="2" t="n">
+        <v>45764</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Training Courses</t>
         </is>
       </c>
-      <c r="E26" t="n">
+      <c r="E26" s="2" t="n">
         <v>3936.39</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>EXP-0026</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2025-07-06</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
+      <c r="B27" s="2" t="n">
+        <v>45844</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Team Lunch</t>
         </is>
       </c>
-      <c r="E27" t="n">
+      <c r="E27" s="2" t="n">
         <v>1461.98</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>EXP-0027</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>2025-09-09</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
+      <c r="B28" s="2" t="n">
+        <v>45909</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Laptops</t>
         </is>
       </c>
-      <c r="E28" t="n">
+      <c r="E28" s="2" t="n">
         <v>3498.13</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>EXP-0028</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>2025-12-20</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
+      <c r="B29" s="2" t="n">
+        <v>46011</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Legal Consultation</t>
         </is>
       </c>
-      <c r="E29" t="n">
+      <c r="E29" s="2" t="n">
         <v>3666</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>EXP-0029</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>2025-08-25</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
+      <c r="B30" s="2" t="n">
+        <v>45894</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Legal Consultation</t>
         </is>
       </c>
-      <c r="E30" t="n">
+      <c r="E30" s="2" t="n">
         <v>3927.64</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>EXP-0030</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>2025-06-14</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
+      <c r="B31" s="2" t="n">
+        <v>45822</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Client Dinner</t>
         </is>
       </c>
-      <c r="E31" t="n">
+      <c r="E31" s="2" t="n">
         <v>3326.26</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>EXP-0031</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>2025-11-20</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
+      <c r="B32" s="2" t="n">
+        <v>45981</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Server Hosting</t>
         </is>
       </c>
-      <c r="E32" t="n">
+      <c r="E32" s="2" t="n">
         <v>2459.02</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>EXP-0032</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
+      <c r="B33" s="2" t="n">
+        <v>46120</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Electricity Bill</t>
         </is>
       </c>
-      <c r="E33" t="n">
+      <c r="E33" s="2" t="n">
         <v>989.99</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>EXP-0033</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>2026-01-20</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
+      <c r="B34" s="2" t="n">
+        <v>46042</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Online Ads</t>
         </is>
       </c>
-      <c r="E34" t="n">
+      <c r="E34" s="2" t="n">
         <v>1127.62</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>EXP-0034</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>2025-04-19</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
+      <c r="B35" s="2" t="n">
+        <v>45766</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Server Hosting</t>
         </is>
       </c>
-      <c r="E35" t="n">
+      <c r="E35" s="2" t="n">
         <v>339.49</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>EXP-0035</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>2025-09-07</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
+      <c r="B36" s="2" t="n">
+        <v>45907</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Airfare</t>
         </is>
       </c>
-      <c r="E36" t="n">
+      <c r="E36" s="2" t="n">
         <v>3691.9</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>EXP-0036</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>2025-10-19</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
+      <c r="B37" s="2" t="n">
+        <v>45949</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E37" t="n">
+      <c r="E37" s="2" t="n">
         <v>351.74</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>EXP-0037</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>2025-11-20</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
+      <c r="B38" s="2" t="n">
+        <v>45981</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E38" t="n">
+      <c r="E38" s="2" t="n">
         <v>1602.34</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>EXP-0038</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
+      <c r="B39" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Airfare</t>
         </is>
       </c>
-      <c r="E39" t="n">
+      <c r="E39" s="2" t="n">
         <v>298.2</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>EXP-0039</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>2025-12-22</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
+      <c r="B40" s="2" t="n">
+        <v>46013</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Client Dinner</t>
         </is>
       </c>
-      <c r="E40" t="n">
+      <c r="E40" s="2" t="n">
         <v>2410.1</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>EXP-0040</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>2025-10-21</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
+      <c r="B41" s="2" t="n">
+        <v>45951</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Software Licenses</t>
         </is>
       </c>
-      <c r="E41" t="n">
+      <c r="E41" s="2" t="n">
         <v>4600.97</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>EXP-0041</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>2026-02-18</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
+      <c r="B42" s="2" t="n">
+        <v>46071</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>Event Sponsorship</t>
         </is>
       </c>
-      <c r="E42" t="n">
+      <c r="E42" s="2" t="n">
         <v>2679.07</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>EXP-0042</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
+      <c r="B43" s="2" t="n">
+        <v>46076</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>Online Ads</t>
         </is>
       </c>
-      <c r="E43" t="n">
+      <c r="E43" s="2" t="n">
         <v>331.55</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>EXP-0043</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>2025-09-29</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
+      <c r="B44" s="2" t="n">
+        <v>45929</v>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E44" t="n">
+      <c r="E44" s="2" t="n">
         <v>2563.75</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>EXP-0044</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>2026-02-21</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
+      <c r="B45" s="2" t="n">
+        <v>46074</v>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>Event Sponsorship</t>
         </is>
       </c>
-      <c r="E45" t="n">
+      <c r="E45" s="2" t="n">
         <v>4264.15</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>EXP-0045</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>2025-10-10</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
+      <c r="B46" s="2" t="n">
+        <v>45940</v>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E46" t="n">
+      <c r="E46" s="2" t="n">
         <v>389.18</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>EXP-0046</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>2025-10-17</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
+      <c r="B47" s="2" t="n">
+        <v>45947</v>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>Software Licenses</t>
         </is>
       </c>
-      <c r="E47" t="n">
+      <c r="E47" s="2" t="n">
         <v>386.41</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>EXP-0047</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>2025-06-06</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
+      <c r="B48" s="2" t="n">
+        <v>45814</v>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Airfare</t>
         </is>
       </c>
-      <c r="E48" t="n">
+      <c r="E48" s="2" t="n">
         <v>4316.01</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>EXP-0048</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>2025-11-27</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
+      <c r="B49" s="2" t="n">
+        <v>45988</v>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>Training Courses</t>
         </is>
       </c>
-      <c r="E49" t="n">
+      <c r="E49" s="2" t="n">
         <v>2048.69</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>EXP-0049</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
+      <c r="B50" s="2" t="n">
+        <v>46101</v>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Legal Consultation</t>
         </is>
       </c>
-      <c r="E50" t="n">
+      <c r="E50" s="2" t="n">
         <v>4710.9</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>EXP-0050</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>2025-08-19</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
+      <c r="B51" s="2" t="n">
+        <v>45888</v>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>Software Licenses</t>
         </is>
       </c>
-      <c r="E51" t="n">
+      <c r="E51" s="2" t="n">
         <v>2869.89</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>EXP-0051</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>2025-07-11</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
+      <c r="B52" s="2" t="n">
+        <v>45849</v>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E52" t="n">
+      <c r="E52" s="2" t="n">
         <v>2915.65</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>EXP-0052</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>2026-02-07</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
+      <c r="B53" s="2" t="n">
+        <v>46060</v>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>Airfare</t>
         </is>
       </c>
-      <c r="E53" t="n">
+      <c r="E53" s="2" t="n">
         <v>246.72</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>EXP-0053</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>2025-09-30</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
+      <c r="B54" s="2" t="n">
+        <v>45930</v>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>Electricity Bill</t>
         </is>
       </c>
-      <c r="E54" t="n">
+      <c r="E54" s="2" t="n">
         <v>455.82</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>EXP-0054</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>2026-03-02</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
+      <c r="B55" s="2" t="n">
+        <v>46083</v>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>Software Licenses</t>
         </is>
       </c>
-      <c r="E55" t="n">
+      <c r="E55" s="2" t="n">
         <v>3304</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>EXP-0055</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>2025-07-03</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
+      <c r="B56" s="2" t="n">
+        <v>45841</v>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Internet Bill</t>
         </is>
       </c>
-      <c r="E56" t="n">
+      <c r="E56" s="2" t="n">
         <v>2847.87</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>EXP-0056</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>2025-11-12</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
+      <c r="B57" s="2" t="n">
+        <v>45973</v>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>Client Dinner</t>
         </is>
       </c>
-      <c r="E57" t="n">
+      <c r="E57" s="2" t="n">
         <v>1616.03</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>EXP-0057</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>2025-05-25</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
+      <c r="B58" s="2" t="n">
+        <v>45802</v>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Airfare</t>
         </is>
       </c>
-      <c r="E58" t="n">
+      <c r="E58" s="2" t="n">
         <v>1340.79</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>EXP-0058</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>2025-05-30</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
+      <c r="B59" s="2" t="n">
+        <v>45807</v>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Online Ads</t>
         </is>
       </c>
-      <c r="E59" t="n">
+      <c r="E59" s="2" t="n">
         <v>3365.14</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>EXP-0059</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>2025-10-08</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
+      <c r="B60" s="2" t="n">
+        <v>45938</v>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E60" t="n">
+      <c r="E60" s="2" t="n">
         <v>1605.21</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>EXP-0060</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>2025-06-20</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
+      <c r="B61" s="2" t="n">
+        <v>45828</v>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Team Lunch</t>
         </is>
       </c>
-      <c r="E61" t="n">
+      <c r="E61" s="2" t="n">
         <v>1364.79</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>EXP-0061</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>2026-01-03</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
+      <c r="B62" s="2" t="n">
+        <v>46025</v>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>Legal Consultation</t>
         </is>
       </c>
-      <c r="E62" t="n">
+      <c r="E62" s="2" t="n">
         <v>697.85</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>EXP-0062</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>2025-04-16</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
+      <c r="B63" s="2" t="n">
+        <v>45763</v>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>Server Hosting</t>
         </is>
       </c>
-      <c r="E63" t="n">
+      <c r="E63" s="2" t="n">
         <v>3245.23</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>EXP-0063</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
+      <c r="B64" s="2" t="n">
+        <v>46088</v>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E64" t="n">
+      <c r="E64" s="2" t="n">
         <v>2313.26</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>EXP-0064</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>2026-03-19</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
+      <c r="B65" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>Online Ads</t>
         </is>
       </c>
-      <c r="E65" t="n">
+      <c r="E65" s="2" t="n">
         <v>4648.64</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>EXP-0065</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>2025-05-08</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
+      <c r="B66" s="2" t="n">
+        <v>45785</v>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>Hotel Accommodation</t>
         </is>
       </c>
-      <c r="E66" t="n">
+      <c r="E66" s="2" t="n">
         <v>4681.88</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>EXP-0066</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>2025-12-16</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
+      <c r="B67" s="2" t="n">
+        <v>46007</v>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>Training Courses</t>
         </is>
       </c>
-      <c r="E67" t="n">
+      <c r="E67" s="2" t="n">
         <v>96.11</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>EXP-0067</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>2025-11-14</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
+      <c r="B68" s="2" t="n">
+        <v>45975</v>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>Electricity Bill</t>
         </is>
       </c>
-      <c r="E68" t="n">
+      <c r="E68" s="2" t="n">
         <v>3124.74</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>EXP-0068</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>2026-03-02</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
+      <c r="B69" s="2" t="n">
+        <v>46083</v>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>Electricity Bill</t>
         </is>
       </c>
-      <c r="E69" t="n">
+      <c r="E69" s="2" t="n">
         <v>2836.82</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>EXP-0069</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>2025-12-13</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
+      <c r="B70" s="2" t="n">
+        <v>46004</v>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>Event Sponsorship</t>
         </is>
       </c>
-      <c r="E70" t="n">
+      <c r="E70" s="2" t="n">
         <v>544.91</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>EXP-0070</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
+      <c r="B71" s="2" t="n">
+        <v>46072</v>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>Event Sponsorship</t>
         </is>
       </c>
-      <c r="E71" t="n">
+      <c r="E71" s="2" t="n">
         <v>2711.29</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" s="2" t="inlineStr">
         <is>
           <t>EXP-0071</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>2025-09-29</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
+      <c r="B72" s="2" t="n">
+        <v>45929</v>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr">
         <is>
           <t>Server Hosting</t>
         </is>
       </c>
-      <c r="E72" t="n">
+      <c r="E72" s="2" t="n">
         <v>2554.13</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" s="2" t="inlineStr">
         <is>
           <t>EXP-0072</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>2025-11-20</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
+      <c r="B73" s="2" t="n">
+        <v>45981</v>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
         <is>
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E73" t="n">
+      <c r="E73" s="2" t="n">
         <v>705.66</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="2" t="inlineStr">
         <is>
           <t>EXP-0073</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>2025-08-22</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
+      <c r="B74" s="2" t="n">
+        <v>45891</v>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D74" s="2" t="inlineStr">
         <is>
           <t>Pantry Supplies</t>
         </is>
       </c>
-      <c r="E74" t="n">
+      <c r="E74" s="2" t="n">
         <v>1777.59</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="2" t="inlineStr">
         <is>
           <t>EXP-0074</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>2025-05-21</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
+      <c r="B75" s="2" t="n">
+        <v>45798</v>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D75" s="2" t="inlineStr">
         <is>
           <t>Server Hosting</t>
         </is>
       </c>
-      <c r="E75" t="n">
+      <c r="E75" s="2" t="n">
         <v>390.52</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="2" t="inlineStr">
         <is>
           <t>EXP-0075</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>2025-10-07</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
+      <c r="B76" s="2" t="n">
+        <v>45937</v>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D76" s="2" t="inlineStr">
         <is>
           <t>Pantry Supplies</t>
         </is>
       </c>
-      <c r="E76" t="n">
+      <c r="E76" s="2" t="n">
         <v>1259.21</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="2" t="inlineStr">
         <is>
           <t>EXP-0076</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>2026-01-18</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
+      <c r="B77" s="2" t="n">
+        <v>46040</v>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D77" s="2" t="inlineStr">
         <is>
           <t>Laptops</t>
         </is>
       </c>
-      <c r="E77" t="n">
+      <c r="E77" s="2" t="n">
         <v>1460.69</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="2" t="inlineStr">
         <is>
           <t>EXP-0077</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>2025-10-04</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
+      <c r="B78" s="2" t="n">
+        <v>45934</v>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D78" s="2" t="inlineStr">
         <is>
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E78" t="n">
+      <c r="E78" s="2" t="n">
         <v>2219.01</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>EXP-0078</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>2025-10-12</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
+      <c r="B79" s="2" t="n">
+        <v>45942</v>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D79" s="2" t="inlineStr">
         <is>
           <t>Airfare</t>
         </is>
       </c>
-      <c r="E79" t="n">
+      <c r="E79" s="2" t="n">
         <v>2738.93</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
+      <c r="A80" s="2" t="inlineStr">
         <is>
           <t>EXP-0079</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>2025-12-25</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
+      <c r="B80" s="2" t="n">
+        <v>46016</v>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="D80" s="2" t="inlineStr">
         <is>
           <t>Airfare</t>
         </is>
       </c>
-      <c r="E80" t="n">
+      <c r="E80" s="2" t="n">
         <v>1547.46</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
+      <c r="A81" s="2" t="inlineStr">
         <is>
           <t>EXP-0080</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>2025-05-03</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
+      <c r="B81" s="2" t="n">
+        <v>45780</v>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D81" s="2" t="inlineStr">
         <is>
           <t>Legal Consultation</t>
         </is>
       </c>
-      <c r="E81" t="n">
+      <c r="E81" s="2" t="n">
         <v>4920.07</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" s="2" t="inlineStr">
         <is>
           <t>EXP-0081</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>2025-11-26</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
+      <c r="B82" s="2" t="n">
+        <v>45987</v>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="D82" s="2" t="inlineStr">
         <is>
           <t>Laptops</t>
         </is>
       </c>
-      <c r="E82" t="n">
+      <c r="E82" s="2" t="n">
         <v>4045.14</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
+      <c r="A83" s="2" t="inlineStr">
         <is>
           <t>EXP-0082</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>2025-04-17</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
+      <c r="B83" s="2" t="n">
+        <v>45764</v>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="D83" s="2" t="inlineStr">
         <is>
           <t>Client Dinner</t>
         </is>
       </c>
-      <c r="E83" t="n">
+      <c r="E83" s="2" t="n">
         <v>2668.26</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
+      <c r="A84" s="2" t="inlineStr">
         <is>
           <t>EXP-0083</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>2025-04-27</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
+      <c r="B84" s="2" t="n">
+        <v>45774</v>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D84" s="2" t="inlineStr">
         <is>
           <t>Laptops</t>
         </is>
       </c>
-      <c r="E84" t="n">
+      <c r="E84" s="2" t="n">
         <v>3355.92</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>EXP-0084</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>2025-05-15</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
+      <c r="B85" s="2" t="n">
+        <v>45792</v>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D85" s="2" t="inlineStr">
         <is>
           <t>Laptops</t>
         </is>
       </c>
-      <c r="E85" t="n">
+      <c r="E85" s="2" t="n">
         <v>2795.28</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="2" t="inlineStr">
         <is>
           <t>EXP-0085</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
+      <c r="B86" s="2" t="n">
+        <v>46087</v>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D86" s="2" t="inlineStr">
         <is>
           <t>Server Hosting</t>
         </is>
       </c>
-      <c r="E86" t="n">
+      <c r="E86" s="2" t="n">
         <v>4662.19</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
+      <c r="A87" s="2" t="inlineStr">
         <is>
           <t>EXP-0086</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>2025-06-04</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
+      <c r="B87" s="2" t="n">
+        <v>45812</v>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D87" s="2" t="inlineStr">
         <is>
           <t>Internet Bill</t>
         </is>
       </c>
-      <c r="E87" t="n">
+      <c r="E87" s="2" t="n">
         <v>562.75</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
+      <c r="A88" s="2" t="inlineStr">
         <is>
           <t>EXP-0087</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>2025-05-21</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
+      <c r="B88" s="2" t="n">
+        <v>45798</v>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D88" s="2" t="inlineStr">
         <is>
           <t>Training Courses</t>
         </is>
       </c>
-      <c r="E88" t="n">
+      <c r="E88" s="2" t="n">
         <v>4396.73</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
+      <c r="A89" s="2" t="inlineStr">
         <is>
           <t>EXP-0088</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>2026-01-14</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
+      <c r="B89" s="2" t="n">
+        <v>46036</v>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D89" s="2" t="inlineStr">
         <is>
           <t>Software Licenses</t>
         </is>
       </c>
-      <c r="E89" t="n">
+      <c r="E89" s="2" t="n">
         <v>1359.11</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
+      <c r="A90" s="2" t="inlineStr">
         <is>
           <t>EXP-0089</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>2025-07-12</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
+      <c r="B90" s="2" t="n">
+        <v>45850</v>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D90" s="2" t="inlineStr">
         <is>
           <t>Legal Consultation</t>
         </is>
       </c>
-      <c r="E90" t="n">
+      <c r="E90" s="2" t="n">
         <v>4454.08</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
+      <c r="A91" s="2" t="inlineStr">
         <is>
           <t>EXP-0090</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>2025-12-07</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
+      <c r="B91" s="2" t="n">
+        <v>45998</v>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="D91" s="2" t="inlineStr">
         <is>
           <t>Legal Consultation</t>
         </is>
       </c>
-      <c r="E91" t="n">
+      <c r="E91" s="2" t="n">
         <v>3724.96</v>
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
+      <c r="A92" s="2" t="inlineStr">
         <is>
           <t>EXP-0091</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>2026-01-18</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
+      <c r="B92" s="2" t="n">
+        <v>46040</v>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="D92" s="2" t="inlineStr">
         <is>
           <t>Legal Consultation</t>
         </is>
       </c>
-      <c r="E92" t="n">
+      <c r="E92" s="2" t="n">
         <v>819.47</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
+      <c r="A93" s="2" t="inlineStr">
         <is>
           <t>EXP-0092</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>2025-08-18</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
+      <c r="B93" s="2" t="n">
+        <v>45887</v>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D93" s="2" t="inlineStr">
         <is>
           <t>Airfare</t>
         </is>
       </c>
-      <c r="E93" t="n">
+      <c r="E93" s="2" t="n">
         <v>1444.69</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
+      <c r="A94" s="2" t="inlineStr">
         <is>
           <t>EXP-0093</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>2025-09-29</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
+      <c r="B94" s="2" t="n">
+        <v>45929</v>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D94" s="2" t="inlineStr">
         <is>
           <t>Software Licenses</t>
         </is>
       </c>
-      <c r="E94" t="n">
+      <c r="E94" s="2" t="n">
         <v>1092.62</v>
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
+      <c r="A95" s="2" t="inlineStr">
         <is>
           <t>EXP-0094</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>2025-11-24</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
+      <c r="B95" s="2" t="n">
+        <v>45985</v>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="D95" s="2" t="inlineStr">
         <is>
           <t>Laptops</t>
         </is>
       </c>
-      <c r="E95" t="n">
+      <c r="E95" s="2" t="n">
         <v>1747.26</v>
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="A96" s="2" t="inlineStr">
         <is>
           <t>EXP-0095</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>2025-05-19</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
+      <c r="B96" s="2" t="n">
+        <v>45796</v>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="D96" s="2" t="inlineStr">
         <is>
           <t>Training Courses</t>
         </is>
       </c>
-      <c r="E96" t="n">
+      <c r="E96" s="2" t="n">
         <v>3453.11</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="A97" s="2" t="inlineStr">
         <is>
           <t>EXP-0096</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>2025-04-24</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
+      <c r="B97" s="2" t="n">
+        <v>45771</v>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr">
+      <c r="D97" s="2" t="inlineStr">
         <is>
           <t>Client Dinner</t>
         </is>
       </c>
-      <c r="E97" t="n">
+      <c r="E97" s="2" t="n">
         <v>4271.92</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
+      <c r="A98" s="2" t="inlineStr">
         <is>
           <t>EXP-0097</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>2025-06-30</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
+      <c r="B98" s="2" t="n">
+        <v>45838</v>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr">
+      <c r="D98" s="2" t="inlineStr">
         <is>
           <t>Pantry Supplies</t>
         </is>
       </c>
-      <c r="E98" t="n">
+      <c r="E98" s="2" t="n">
         <v>2551.77</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
+      <c r="A99" s="2" t="inlineStr">
         <is>
           <t>EXP-0098</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>2025-12-20</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
+      <c r="B99" s="2" t="n">
+        <v>46011</v>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr">
+      <c r="D99" s="2" t="inlineStr">
         <is>
           <t>Internet Bill</t>
         </is>
       </c>
-      <c r="E99" t="n">
+      <c r="E99" s="2" t="n">
         <v>1293.05</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
+      <c r="A100" s="2" t="inlineStr">
         <is>
           <t>EXP-0099</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>2025-04-26</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
+      <c r="B100" s="2" t="n">
+        <v>45773</v>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr">
+      <c r="D100" s="2" t="inlineStr">
         <is>
           <t>Airfare</t>
         </is>
       </c>
-      <c r="E100" t="n">
+      <c r="E100" s="2" t="n">
         <v>4545.39</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
+      <c r="A101" s="2" t="inlineStr">
         <is>
           <t>EXP-0100</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>2025-10-27</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
+      <c r="B101" s="2" t="n">
+        <v>45957</v>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr">
+      <c r="D101" s="2" t="inlineStr">
         <is>
           <t>Office Supplies</t>
         </is>
       </c>
-      <c r="E101" t="n">
+      <c r="E101" s="2" t="n">
         <v>301.45</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>EXP12345</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Random Item</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>123.45</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -3092,81 +2831,94 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Amount ($)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>24351.8</v>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>24351.8</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>48229.62</v>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>48229.62</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>28037.96</v>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>28037.96</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>37609.16</v>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>37609.16</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>54489.82</v>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>54489.82</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>40553.62</v>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>40553.62</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>